<commit_message>
Cat Shelter: update BOM v4 and v1.1 firmware
</commit_message>
<xml_diff>
--- a/docs/Cat_Shelter_BOM_v4.xlsx
+++ b/docs/Cat_Shelter_BOM_v4.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Locked Decisions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="145621"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -71,9 +72,6 @@
     <t>BLE required from day one; Micro-USB for programming (USB-C not required); on-board LiPo charger present but not used in field.</t>
   </si>
   <si>
-    <t>Storage</t>
-  </si>
-  <si>
     <t>Non-volatile memory breakout (SPI FRAM 256KB)</t>
   </si>
   <si>
@@ -423,6 +421,9 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Data Storage</t>
   </si>
 </sst>
 </file>
@@ -518,7 +519,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -579,6 +580,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -785,13 +789,13 @@
     <col min="9" max="10" width="11.140625" style="9" customWidth="1"/>
     <col min="11" max="11" width="58.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" style="4" customWidth="1"/>
-    <col min="13" max="13" width="46" style="2" customWidth="1"/>
+    <col min="13" max="13" width="47.140625" style="2" customWidth="1"/>
     <col min="14" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1" s="12" t="s">
         <v>0</v>
@@ -815,10 +819,10 @@
         <v>6</v>
       </c>
       <c r="I1" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="J1" s="19" t="s">
         <v>129</v>
-      </c>
-      <c r="J1" s="19" t="s">
-        <v>130</v>
       </c>
       <c r="K1" s="12" t="s">
         <v>7</v>
@@ -859,7 +863,7 @@
         <v>24.95</v>
       </c>
       <c r="J2" s="16">
-        <f>IF(OR(I2="",H2=""),"",H2*I2)</f>
+        <f t="shared" ref="J2:J9" si="0">IF(OR(I2="",H2=""),"",H2*I2)</f>
         <v>24.95</v>
       </c>
       <c r="K2" s="17" t="s">
@@ -877,22 +881,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C3" s="18" t="s">
         <v>18</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>19</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="G3" s="15" t="s">
         <v>21</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>22</v>
       </c>
       <c r="H3" s="15">
         <v>1</v>
@@ -901,17 +905,17 @@
         <v>12.95</v>
       </c>
       <c r="J3" s="16">
-        <f>IF(OR(I3="",H3=""),"",H3*I3)</f>
+        <f t="shared" si="0"/>
         <v>12.95</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L3" s="14" t="s">
         <v>16</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -919,22 +923,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="18" t="s">
         <v>25</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>26</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="G4" s="15" t="s">
         <v>28</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>29</v>
       </c>
       <c r="H4" s="15">
         <v>1</v>
@@ -943,17 +947,17 @@
         <v>17.5</v>
       </c>
       <c r="J4" s="16">
-        <f>IF(OR(I4="",H4=""),"",H4*I4)</f>
+        <f t="shared" si="0"/>
         <v>17.5</v>
       </c>
       <c r="K4" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="14" t="s">
+      <c r="M4" s="18" t="s">
         <v>31</v>
-      </c>
-      <c r="M4" s="18" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -961,22 +965,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E5" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="G5" s="15" t="s">
         <v>35</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>36</v>
       </c>
       <c r="H5" s="15">
         <v>1</v>
@@ -985,17 +989,17 @@
         <v>0.95</v>
       </c>
       <c r="J5" s="16">
-        <f>IF(OR(I5="",H5=""),"",H5*I5)</f>
+        <f t="shared" si="0"/>
         <v>0.95</v>
       </c>
       <c r="K5" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M5" s="18" t="s">
         <v>37</v>
-      </c>
-      <c r="L5" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="M5" s="18" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -1003,22 +1007,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="18" t="s">
         <v>39</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>40</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="G6" s="15" t="s">
         <v>42</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>43</v>
       </c>
       <c r="H6" s="15">
         <v>2</v>
@@ -1026,18 +1030,18 @@
       <c r="I6" s="16">
         <v>9.9499999999999993</v>
       </c>
-      <c r="J6" s="16">
-        <f>IF(OR(I6="",H6=""),"",H6*I6)</f>
+      <c r="J6" s="21">
+        <f t="shared" si="0"/>
         <v>19.899999999999999</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L6" s="14" t="s">
         <v>16</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -1045,22 +1049,22 @@
         <v>8</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H7" s="15">
         <v>1</v>
@@ -1069,17 +1073,17 @@
         <v>2.5</v>
       </c>
       <c r="J7" s="16">
-        <f>IF(OR(I7="",H7=""),"",H7*I7)</f>
+        <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
       <c r="K7" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M7" s="18" t="s">
         <v>58</v>
-      </c>
-      <c r="L7" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="M7" s="18" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -1087,22 +1091,22 @@
         <v>10</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>65</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>66</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H8" s="15">
         <v>0</v>
@@ -1111,17 +1115,17 @@
         <v>9.9499999999999993</v>
       </c>
       <c r="J8" s="16">
-        <f>IF(OR(I8="",H8=""),"",H8*I8)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L8" s="14" t="s">
         <v>16</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -1129,22 +1133,22 @@
         <v>12</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="18" t="s">
         <v>74</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>75</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H9" s="15">
         <v>1</v>
@@ -1153,17 +1157,17 @@
         <v>2.95</v>
       </c>
       <c r="J9" s="16">
-        <f>IF(OR(I9="",H9=""),"",H9*I9)</f>
+        <f t="shared" si="0"/>
         <v>2.95</v>
       </c>
       <c r="K9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M9" s="18" t="s">
         <v>77</v>
-      </c>
-      <c r="L9" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="M9" s="18" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1171,13 +1175,13 @@
         <v>19</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E10" s="15"/>
       <c r="F10" s="14"/>
@@ -1188,7 +1192,7 @@
         <v>13.82</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L10" s="14"/>
       <c r="M10" s="18"/>
@@ -1199,34 +1203,34 @@
         <v>95.52000000000001</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J12" s="8"/>
       <c r="K12" s="5"/>
     </row>
-    <row r="14" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="12">
         <v>6</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H14" s="15">
         <v>0</v>
@@ -1235,17 +1239,17 @@
         <v>0.75</v>
       </c>
       <c r="J14" s="16">
-        <f>IF(OR(I14="",H14=""),"",H14*I14)</f>
+        <f t="shared" ref="J14:J23" si="1">IF(OR(I14="",H14=""),"",H14*I14)</f>
         <v>0</v>
       </c>
       <c r="K14" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="L14" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="L14" s="14" t="s">
+      <c r="M14" s="18" t="s">
         <v>49</v>
-      </c>
-      <c r="M14" s="18" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -1253,22 +1257,22 @@
         <v>7</v>
       </c>
       <c r="B15" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="18" t="s">
         <v>51</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>52</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H15" s="15">
         <v>0</v>
@@ -1277,17 +1281,17 @@
         <v>19.95</v>
       </c>
       <c r="J15" s="16">
-        <f>IF(OR(I15="",H15=""),"",H15*I15)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K15" s="17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L15" s="14" t="s">
         <v>16</v>
       </c>
       <c r="M15" s="18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -1295,22 +1299,22 @@
         <v>9</v>
       </c>
       <c r="B16" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="18" t="s">
         <v>60</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>61</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F16" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H16" s="15">
         <v>0</v>
@@ -1319,17 +1323,17 @@
         <v>5.95</v>
       </c>
       <c r="J16" s="16">
-        <f>IF(OR(I16="",H16=""),"",H16*I16)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K16" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="L16" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M16" s="18" t="s">
         <v>63</v>
-      </c>
-      <c r="L16" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="M16" s="18" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -1337,22 +1341,22 @@
         <v>11</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H17" s="15">
         <v>0</v>
@@ -1361,17 +1365,17 @@
         <v>1.95</v>
       </c>
       <c r="J17" s="16">
-        <f>IF(OR(I17="",H17=""),"",H17*I17)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K17" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="L17" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="M17" s="18" t="s">
         <v>72</v>
-      </c>
-      <c r="L17" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="M17" s="18" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -1379,22 +1383,22 @@
         <v>13</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F18" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H18" s="15">
         <v>0</v>
@@ -1403,17 +1407,17 @@
         <v>2.95</v>
       </c>
       <c r="J18" s="16">
-        <f>IF(OR(I18="",H18=""),"",H18*I18)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K18" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="L18" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="M18" s="18" t="s">
         <v>81</v>
-      </c>
-      <c r="L18" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="M18" s="18" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -1421,22 +1425,22 @@
         <v>14</v>
       </c>
       <c r="B19" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="18" t="s">
         <v>83</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>84</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H19" s="15">
         <v>0</v>
@@ -1445,17 +1449,17 @@
         <v>8.5</v>
       </c>
       <c r="J19" s="16">
-        <f>IF(OR(I19="",H19=""),"",H19*I19)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K19" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="L19" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M19" s="18" t="s">
         <v>86</v>
-      </c>
-      <c r="L19" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="M19" s="18" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -1463,22 +1467,22 @@
         <v>15</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H20" s="15">
         <v>0</v>
@@ -1487,17 +1491,17 @@
         <v>4.95</v>
       </c>
       <c r="J20" s="16">
-        <f>IF(OR(I20="",H20=""),"",H20*I20)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K20" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="L20" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="M20" s="18" t="s">
         <v>90</v>
-      </c>
-      <c r="L20" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="M20" s="18" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -1505,22 +1509,22 @@
         <v>16</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>92</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>93</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H21" s="15">
         <v>0</v>
@@ -1529,17 +1533,17 @@
         <v>4.95</v>
       </c>
       <c r="J21" s="16">
-        <f>IF(OR(I21="",H21=""),"",H21*I21)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K21" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="L21" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M21" s="18" t="s">
         <v>95</v>
-      </c>
-      <c r="L21" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="M21" s="18" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -1547,22 +1551,22 @@
         <v>17</v>
       </c>
       <c r="B22" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="C22" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="D22" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="E22" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="F22" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="G22" s="15" t="s">
         <v>101</v>
-      </c>
-      <c r="G22" s="15" t="s">
-        <v>102</v>
       </c>
       <c r="H22" s="15">
         <v>0</v>
@@ -1571,17 +1575,17 @@
         <v>5.93</v>
       </c>
       <c r="J22" s="16">
-        <f>IF(OR(I22="",H22=""),"",H22*I22)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K22" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="L22" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="M22" s="18" t="s">
         <v>103</v>
-      </c>
-      <c r="L22" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="M22" s="18" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -1589,22 +1593,22 @@
         <v>18</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C23" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="E23" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="D23" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="E23" s="15" t="s">
+      <c r="F23" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="G23" s="15" t="s">
         <v>106</v>
-      </c>
-      <c r="F23" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="G23" s="15" t="s">
-        <v>107</v>
       </c>
       <c r="H23" s="15">
         <v>0</v>
@@ -1613,17 +1617,17 @@
         <v>1.24</v>
       </c>
       <c r="J23" s="16">
-        <f>IF(OR(I23="",H23=""),"",H23*I23)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K23" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="L23" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="M23" s="18" t="s">
         <v>108</v>
-      </c>
-      <c r="L23" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="M23" s="18" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -1682,53 +1686,53 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1736,27 +1740,27 @@
     </row>
     <row r="13" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1764,22 +1768,22 @@
     </row>
     <row r="19" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>